<commit_message>
Switch to new brochure: real layouts matched to unit areas
- Replace layouts/renders/master-plan with ion brochure Final assets
- 15 real floor-plan layouts; inventory areas = actual plan areas so the
  selected unit always shows its matching layout
- Aerial (labeled) master plan with re-derived building pins
- Prices computed per-m2 from the published price list
- Remove old prime-ions brochure assets

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/deliverables/Ion-Phase2-Units-DEMO.xlsx
+++ b/assets/deliverables/Ion-Phase2-Units-DEMO.xlsx
@@ -457,13 +457,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E2">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="F2" t="str">
         <v>Street</v>
       </c>
       <c r="G2">
-        <v>8687195</v>
+        <v>7932192</v>
       </c>
       <c r="H2" t="str">
         <v>Fully Finished</v>
@@ -472,7 +472,7 @@
         <v>Available</v>
       </c>
       <c r="J2" t="str">
-        <v>3br-b</v>
+        <v>3br-t7</v>
       </c>
     </row>
     <row r="3">
@@ -486,16 +486,16 @@
         <v>2nd</v>
       </c>
       <c r="D3" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E3">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F3" t="str">
         <v>Landscape</v>
       </c>
       <c r="G3">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H3" t="str">
         <v>Fully Finished</v>
@@ -504,7 +504,7 @@
         <v>Available</v>
       </c>
       <c r="J3" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="4">
@@ -518,16 +518,16 @@
         <v>4th</v>
       </c>
       <c r="D4" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E4">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="F4" t="str">
         <v>Garden</v>
       </c>
       <c r="G4">
-        <v>8888055</v>
+        <v>11348590</v>
       </c>
       <c r="H4" t="str">
         <v>Fully Finished</v>
@@ -536,7 +536,7 @@
         <v>Available</v>
       </c>
       <c r="J4" t="str">
-        <v>3br-c</v>
+        <v>4br-t1</v>
       </c>
     </row>
     <row r="5">
@@ -550,16 +550,16 @@
         <v>4th</v>
       </c>
       <c r="D5" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E5">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F5" t="str">
         <v>Pool</v>
       </c>
       <c r="G5">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H5" t="str">
         <v>Fully Finished</v>
@@ -568,7 +568,7 @@
         <v>Available</v>
       </c>
       <c r="J5" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="6">
@@ -585,13 +585,13 @@
         <v>4 Bedrooms</v>
       </c>
       <c r="E6">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="F6" t="str">
         <v>Landscape</v>
       </c>
       <c r="G6">
-        <v>8988485</v>
+        <v>9892355</v>
       </c>
       <c r="H6" t="str">
         <v>Fully Finished</v>
@@ -600,7 +600,7 @@
         <v>Available</v>
       </c>
       <c r="J6" t="str">
-        <v>4br-a</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="7">
@@ -614,16 +614,16 @@
         <v>2nd</v>
       </c>
       <c r="D7" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E7">
-        <v>183</v>
+        <v>200</v>
       </c>
       <c r="F7" t="str">
         <v>Landscape</v>
       </c>
       <c r="G7">
-        <v>9017760</v>
+        <v>10043000</v>
       </c>
       <c r="H7" t="str">
         <v>Fully Finished</v>
@@ -632,7 +632,7 @@
         <v>Available</v>
       </c>
       <c r="J7" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="8">
@@ -646,16 +646,16 @@
         <v>2nd</v>
       </c>
       <c r="D8" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E8">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F8" t="str">
         <v>Pool</v>
       </c>
       <c r="G8">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H8" t="str">
         <v>Fully Finished</v>
@@ -664,7 +664,7 @@
         <v>Available</v>
       </c>
       <c r="J8" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="9">
@@ -681,13 +681,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E9">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="F9" t="str">
         <v>Garden</v>
       </c>
       <c r="G9">
-        <v>5852835</v>
+        <v>6422580</v>
       </c>
       <c r="H9" t="str">
         <v>Fully Finished</v>
@@ -696,7 +696,7 @@
         <v>Available</v>
       </c>
       <c r="J9" t="str">
-        <v>2br-a</v>
+        <v>2br-t1</v>
       </c>
     </row>
     <row r="10">
@@ -710,16 +710,16 @@
         <v>2nd</v>
       </c>
       <c r="D10" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E10">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="F10" t="str">
         <v>Street</v>
       </c>
       <c r="G10">
-        <v>9478811</v>
+        <v>10043000</v>
       </c>
       <c r="H10" t="str">
         <v>Fully Finished</v>
@@ -728,7 +728,7 @@
         <v>Available</v>
       </c>
       <c r="J10" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="11">
@@ -742,16 +742,16 @@
         <v>5th</v>
       </c>
       <c r="D11" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E11">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F11" t="str">
         <v>Garden</v>
       </c>
       <c r="G11">
-        <v>9478811</v>
+        <v>9892355</v>
       </c>
       <c r="H11" t="str">
         <v>Fully Finished</v>
@@ -760,7 +760,7 @@
         <v>Available</v>
       </c>
       <c r="J11" t="str">
-        <v>3br-d</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="12">
@@ -777,13 +777,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E12">
-        <v>140</v>
+        <v>197</v>
       </c>
       <c r="F12" t="str">
         <v>Landscape</v>
       </c>
       <c r="G12">
-        <v>6082163</v>
+        <v>9827936</v>
       </c>
       <c r="H12" t="str">
         <v>Fully Finished</v>
@@ -792,7 +792,7 @@
         <v>Available</v>
       </c>
       <c r="J12" t="str">
-        <v>3br-a</v>
+        <v>3br-t5</v>
       </c>
     </row>
     <row r="13">
@@ -806,16 +806,16 @@
         <v>4th</v>
       </c>
       <c r="D13" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E13">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F13" t="str">
         <v>Pool</v>
       </c>
       <c r="G13">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H13" t="str">
         <v>Fully Finished</v>
@@ -824,7 +824,7 @@
         <v>Available</v>
       </c>
       <c r="J13" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="14">
@@ -838,16 +838,16 @@
         <v>6th</v>
       </c>
       <c r="D14" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E14">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="F14" t="str">
         <v>Garden</v>
       </c>
       <c r="G14">
-        <v>8888055</v>
+        <v>11348590</v>
       </c>
       <c r="H14" t="str">
         <v>Fully Finished</v>
@@ -856,7 +856,7 @@
         <v>Available</v>
       </c>
       <c r="J14" t="str">
-        <v>3br-c</v>
+        <v>4br-t1</v>
       </c>
     </row>
     <row r="15">
@@ -873,13 +873,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E15">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="F15" t="str">
         <v>Landscape</v>
       </c>
       <c r="G15">
-        <v>7380720</v>
+        <v>9129504</v>
       </c>
       <c r="H15" t="str">
         <v>Fully Finished</v>
@@ -888,7 +888,7 @@
         <v>Available</v>
       </c>
       <c r="J15" t="str">
-        <v>3br-a</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="16">
@@ -902,16 +902,16 @@
         <v>1st</v>
       </c>
       <c r="D16" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E16">
-        <v>183</v>
+        <v>200</v>
       </c>
       <c r="F16" t="str">
         <v>Landscape</v>
       </c>
       <c r="G16">
-        <v>9017760</v>
+        <v>10043000</v>
       </c>
       <c r="H16" t="str">
         <v>Fully Finished</v>
@@ -920,7 +920,7 @@
         <v>Available</v>
       </c>
       <c r="J16" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="17">
@@ -934,16 +934,16 @@
         <v>3rd</v>
       </c>
       <c r="D17" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E17">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F17" t="str">
         <v>Landscape</v>
       </c>
       <c r="G17">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H17" t="str">
         <v>Fully Finished</v>
@@ -952,7 +952,7 @@
         <v>Available</v>
       </c>
       <c r="J17" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="18">
@@ -966,16 +966,16 @@
         <v>5th</v>
       </c>
       <c r="D18" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E18">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F18" t="str">
         <v>Garden</v>
       </c>
       <c r="G18">
-        <v>9017760</v>
+        <v>11147730</v>
       </c>
       <c r="H18" t="str">
         <v>Fully Finished</v>
@@ -984,7 +984,7 @@
         <v>Available</v>
       </c>
       <c r="J18" t="str">
-        <v>3br-d</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="19">
@@ -998,16 +998,16 @@
         <v>5th</v>
       </c>
       <c r="D19" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E19">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="F19" t="str">
         <v>Pool</v>
       </c>
       <c r="G19">
-        <v>6681555</v>
+        <v>8431072</v>
       </c>
       <c r="H19" t="str">
         <v>Fully Finished</v>
@@ -1016,7 +1016,7 @@
         <v>Available</v>
       </c>
       <c r="J19" t="str">
-        <v>2br-b</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="20">
@@ -1033,13 +1033,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E20">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F20" t="str">
         <v>Street</v>
       </c>
       <c r="G20">
-        <v>6111810</v>
+        <v>6370785</v>
       </c>
       <c r="H20" t="str">
         <v>Fully Finished</v>
@@ -1048,7 +1048,7 @@
         <v>Available</v>
       </c>
       <c r="J20" t="str">
-        <v>2br-a</v>
+        <v>2br-t3</v>
       </c>
     </row>
     <row r="21">
@@ -1065,13 +1065,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E21">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="F21" t="str">
         <v>Garden</v>
       </c>
       <c r="G21">
-        <v>5852835</v>
+        <v>7251300</v>
       </c>
       <c r="H21" t="str">
         <v>Fully Finished</v>
@@ -1080,7 +1080,7 @@
         <v>Available</v>
       </c>
       <c r="J21" t="str">
-        <v>2br-a</v>
+        <v>2br-t2</v>
       </c>
     </row>
     <row r="22">
@@ -1094,16 +1094,16 @@
         <v>6th</v>
       </c>
       <c r="D22" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E22">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F22" t="str">
         <v>Street</v>
       </c>
       <c r="G22">
-        <v>9017760</v>
+        <v>11147730</v>
       </c>
       <c r="H22" t="str">
         <v>Fully Finished</v>
@@ -1112,7 +1112,7 @@
         <v>Available</v>
       </c>
       <c r="J22" t="str">
-        <v>3br-d</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="23">
@@ -1129,13 +1129,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E23">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F23" t="str">
         <v>Street</v>
       </c>
       <c r="G23">
-        <v>6111810</v>
+        <v>6370785</v>
       </c>
       <c r="H23" t="str">
         <v>Fully Finished</v>
@@ -1144,7 +1144,7 @@
         <v>Available</v>
       </c>
       <c r="J23" t="str">
-        <v>2br-a</v>
+        <v>2br-t3</v>
       </c>
     </row>
     <row r="24">
@@ -1158,16 +1158,16 @@
         <v>7th</v>
       </c>
       <c r="D24" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E24">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F24" t="str">
         <v>Garden</v>
       </c>
       <c r="G24">
-        <v>9478811</v>
+        <v>9892355</v>
       </c>
       <c r="H24" t="str">
         <v>Fully Finished</v>
@@ -1176,7 +1176,7 @@
         <v>Available</v>
       </c>
       <c r="J24" t="str">
-        <v>3br-d</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="25">
@@ -1193,13 +1193,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E25">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F25" t="str">
         <v>Landscape</v>
       </c>
       <c r="G25">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H25" t="str">
         <v>Fully Finished</v>
@@ -1208,7 +1208,7 @@
         <v>Available</v>
       </c>
       <c r="J25" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="26">
@@ -1222,16 +1222,16 @@
         <v>6th</v>
       </c>
       <c r="D26" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E26">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F26" t="str">
         <v>Landscape</v>
       </c>
       <c r="G26">
-        <v>9017760</v>
+        <v>11147730</v>
       </c>
       <c r="H26" t="str">
         <v>Fully Finished</v>
@@ -1240,7 +1240,7 @@
         <v>Available</v>
       </c>
       <c r="J26" t="str">
-        <v>3br-d</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="27">
@@ -1257,13 +1257,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E27">
-        <v>153</v>
+        <v>197</v>
       </c>
       <c r="F27" t="str">
         <v>Street</v>
       </c>
       <c r="G27">
-        <v>7380720</v>
+        <v>9827936</v>
       </c>
       <c r="H27" t="str">
         <v>Fully Finished</v>
@@ -1272,7 +1272,7 @@
         <v>Available</v>
       </c>
       <c r="J27" t="str">
-        <v>3br-a</v>
+        <v>3br-t5</v>
       </c>
     </row>
     <row r="28">
@@ -1286,16 +1286,16 @@
         <v>2nd</v>
       </c>
       <c r="D28" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E28">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F28" t="str">
         <v>Landscape</v>
       </c>
       <c r="G28">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H28" t="str">
         <v>Fully Finished</v>
@@ -1304,7 +1304,7 @@
         <v>Available</v>
       </c>
       <c r="J28" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="29">
@@ -1318,16 +1318,16 @@
         <v>6th</v>
       </c>
       <c r="D29" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E29">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F29" t="str">
         <v>Landscape</v>
       </c>
       <c r="G29">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H29" t="str">
         <v>Fully Finished</v>
@@ -1336,7 +1336,7 @@
         <v>Available</v>
       </c>
       <c r="J29" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="30">
@@ -1350,16 +1350,16 @@
         <v>5th</v>
       </c>
       <c r="D30" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E30">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F30" t="str">
         <v>Landscape</v>
       </c>
       <c r="G30">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H30" t="str">
         <v>Fully Finished</v>
@@ -1368,7 +1368,7 @@
         <v>Available</v>
       </c>
       <c r="J30" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="31">
@@ -1382,16 +1382,16 @@
         <v>5th</v>
       </c>
       <c r="D31" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E31">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F31" t="str">
         <v>Street</v>
       </c>
       <c r="G31">
-        <v>9017760</v>
+        <v>11147730</v>
       </c>
       <c r="H31" t="str">
         <v>Fully Finished</v>
@@ -1400,7 +1400,7 @@
         <v>Available</v>
       </c>
       <c r="J31" t="str">
-        <v>3br-d</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="32">
@@ -1417,13 +1417,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E32">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="F32" t="str">
         <v>Landscape</v>
       </c>
       <c r="G32">
-        <v>8687195</v>
+        <v>7932192</v>
       </c>
       <c r="H32" t="str">
         <v>Fully Finished</v>
@@ -1432,7 +1432,7 @@
         <v>Available</v>
       </c>
       <c r="J32" t="str">
-        <v>3br-b</v>
+        <v>3br-t7</v>
       </c>
     </row>
     <row r="33">
@@ -1446,16 +1446,16 @@
         <v>4th</v>
       </c>
       <c r="D33" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E33">
-        <v>183</v>
+        <v>200</v>
       </c>
       <c r="F33" t="str">
         <v>Street</v>
       </c>
       <c r="G33">
-        <v>9017760</v>
+        <v>10043000</v>
       </c>
       <c r="H33" t="str">
         <v>Fully Finished</v>
@@ -1464,7 +1464,7 @@
         <v>Available</v>
       </c>
       <c r="J33" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="34">
@@ -1481,13 +1481,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E34">
-        <v>140</v>
+        <v>197</v>
       </c>
       <c r="F34" t="str">
         <v>Garden</v>
       </c>
       <c r="G34">
-        <v>6082163</v>
+        <v>9827936</v>
       </c>
       <c r="H34" t="str">
         <v>Fully Finished</v>
@@ -1496,7 +1496,7 @@
         <v>Available</v>
       </c>
       <c r="J34" t="str">
-        <v>3br-a</v>
+        <v>3br-t5</v>
       </c>
     </row>
     <row r="35">
@@ -1513,13 +1513,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E35">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F35" t="str">
         <v>Garden</v>
       </c>
       <c r="G35">
-        <v>6441058</v>
+        <v>6370785</v>
       </c>
       <c r="H35" t="str">
         <v>Fully Finished</v>
@@ -1528,7 +1528,7 @@
         <v>Available</v>
       </c>
       <c r="J35" t="str">
-        <v>2br-b</v>
+        <v>2br-t3</v>
       </c>
     </row>
     <row r="36">
@@ -1542,16 +1542,16 @@
         <v>2nd</v>
       </c>
       <c r="D36" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E36">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="F36" t="str">
         <v>Landscape</v>
       </c>
       <c r="G36">
-        <v>8888055</v>
+        <v>11348590</v>
       </c>
       <c r="H36" t="str">
         <v>Fully Finished</v>
@@ -1560,7 +1560,7 @@
         <v>Available</v>
       </c>
       <c r="J36" t="str">
-        <v>3br-c</v>
+        <v>4br-t1</v>
       </c>
     </row>
     <row r="37">
@@ -1577,13 +1577,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E37">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="F37" t="str">
         <v>Pool</v>
       </c>
       <c r="G37">
-        <v>6111810</v>
+        <v>7251300</v>
       </c>
       <c r="H37" t="str">
         <v>Fully Finished</v>
@@ -1592,7 +1592,7 @@
         <v>Available</v>
       </c>
       <c r="J37" t="str">
-        <v>2br-a</v>
+        <v>2br-t2</v>
       </c>
     </row>
     <row r="38">
@@ -1606,16 +1606,16 @@
         <v>3rd</v>
       </c>
       <c r="D38" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E38">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="F38" t="str">
         <v>Landscape</v>
       </c>
       <c r="G38">
-        <v>8888055</v>
+        <v>11348590</v>
       </c>
       <c r="H38" t="str">
         <v>Fully Finished</v>
@@ -1624,7 +1624,7 @@
         <v>Available</v>
       </c>
       <c r="J38" t="str">
-        <v>3br-c</v>
+        <v>4br-t1</v>
       </c>
     </row>
     <row r="39">
@@ -1641,13 +1641,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E39">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="F39" t="str">
         <v>Garden</v>
       </c>
       <c r="G39">
-        <v>8687195</v>
+        <v>7932192</v>
       </c>
       <c r="H39" t="str">
         <v>Fully Finished</v>
@@ -1656,7 +1656,7 @@
         <v>Available</v>
       </c>
       <c r="J39" t="str">
-        <v>3br-b</v>
+        <v>3br-t7</v>
       </c>
     </row>
     <row r="40">
@@ -1670,16 +1670,16 @@
         <v>3rd</v>
       </c>
       <c r="D40" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E40">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F40" t="str">
         <v>Landscape</v>
       </c>
       <c r="G40">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H40" t="str">
         <v>Fully Finished</v>
@@ -1688,7 +1688,7 @@
         <v>Available</v>
       </c>
       <c r="J40" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="41">
@@ -1705,13 +1705,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E41">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F41" t="str">
         <v>Street</v>
       </c>
       <c r="G41">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H41" t="str">
         <v>Fully Finished</v>
@@ -1720,7 +1720,7 @@
         <v>Available</v>
       </c>
       <c r="J41" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="42">
@@ -1734,16 +1734,16 @@
         <v>7th</v>
       </c>
       <c r="D42" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E42">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F42" t="str">
         <v>Pool</v>
       </c>
       <c r="G42">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H42" t="str">
         <v>Fully Finished</v>
@@ -1752,7 +1752,7 @@
         <v>Available</v>
       </c>
       <c r="J42" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="43">
@@ -1769,13 +1769,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E43">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="F43" t="str">
         <v>Street</v>
       </c>
       <c r="G43">
-        <v>8687195</v>
+        <v>7932192</v>
       </c>
       <c r="H43" t="str">
         <v>Fully Finished</v>
@@ -1784,7 +1784,7 @@
         <v>Available</v>
       </c>
       <c r="J43" t="str">
-        <v>3br-b</v>
+        <v>3br-t7</v>
       </c>
     </row>
     <row r="44">
@@ -1801,13 +1801,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E44">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="F44" t="str">
         <v>Garden</v>
       </c>
       <c r="G44">
-        <v>5852835</v>
+        <v>6422580</v>
       </c>
       <c r="H44" t="str">
         <v>Fully Finished</v>
@@ -1816,7 +1816,7 @@
         <v>Available</v>
       </c>
       <c r="J44" t="str">
-        <v>2br-a</v>
+        <v>2br-t1</v>
       </c>
     </row>
     <row r="45">
@@ -1833,13 +1833,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E45">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="F45" t="str">
         <v>Pool</v>
       </c>
       <c r="G45">
-        <v>7380720</v>
+        <v>9129504</v>
       </c>
       <c r="H45" t="str">
         <v>Fully Finished</v>
@@ -1848,7 +1848,7 @@
         <v>Available</v>
       </c>
       <c r="J45" t="str">
-        <v>3br-a</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="46">
@@ -1862,16 +1862,16 @@
         <v>4th</v>
       </c>
       <c r="D46" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E46">
-        <v>124</v>
+        <v>190</v>
       </c>
       <c r="F46" t="str">
         <v>Garden</v>
       </c>
       <c r="G46">
-        <v>6441058</v>
+        <v>9478720</v>
       </c>
       <c r="H46" t="str">
         <v>Fully Finished</v>
@@ -1880,7 +1880,7 @@
         <v>Available</v>
       </c>
       <c r="J46" t="str">
-        <v>2br-b</v>
+        <v>3br-t1</v>
       </c>
     </row>
     <row r="47">
@@ -1897,13 +1897,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E47">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="F47" t="str">
         <v>Street</v>
       </c>
       <c r="G47">
-        <v>8687195</v>
+        <v>9129504</v>
       </c>
       <c r="H47" t="str">
         <v>Fully Finished</v>
@@ -1912,7 +1912,7 @@
         <v>Available</v>
       </c>
       <c r="J47" t="str">
-        <v>3br-b</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="48">
@@ -1926,16 +1926,16 @@
         <v>2nd</v>
       </c>
       <c r="D48" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E48">
-        <v>177</v>
+        <v>222</v>
       </c>
       <c r="F48" t="str">
         <v>Landscape</v>
       </c>
       <c r="G48">
-        <v>8888055</v>
+        <v>11147730</v>
       </c>
       <c r="H48" t="str">
         <v>Fully Finished</v>
@@ -1944,7 +1944,7 @@
         <v>Available</v>
       </c>
       <c r="J48" t="str">
-        <v>3br-c</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="49">
@@ -1961,13 +1961,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E49">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="F49" t="str">
         <v>Garden</v>
       </c>
       <c r="G49">
-        <v>7380720</v>
+        <v>9129504</v>
       </c>
       <c r="H49" t="str">
         <v>Fully Finished</v>
@@ -1976,7 +1976,7 @@
         <v>Available</v>
       </c>
       <c r="J49" t="str">
-        <v>3br-a</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="50">
@@ -1993,13 +1993,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E50">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="F50" t="str">
         <v>Pool</v>
       </c>
       <c r="G50">
-        <v>7380720</v>
+        <v>9129504</v>
       </c>
       <c r="H50" t="str">
         <v>Fully Finished</v>
@@ -2008,7 +2008,7 @@
         <v>Available</v>
       </c>
       <c r="J50" t="str">
-        <v>3br-a</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="51">
@@ -2022,16 +2022,16 @@
         <v>2nd</v>
       </c>
       <c r="D51" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E51">
-        <v>124</v>
+        <v>190</v>
       </c>
       <c r="F51" t="str">
         <v>Street</v>
       </c>
       <c r="G51">
-        <v>6441058</v>
+        <v>9478720</v>
       </c>
       <c r="H51" t="str">
         <v>Fully Finished</v>
@@ -2040,7 +2040,7 @@
         <v>Available</v>
       </c>
       <c r="J51" t="str">
-        <v>2br-b</v>
+        <v>3br-t1</v>
       </c>
     </row>
     <row r="52">
@@ -2057,13 +2057,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E52">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F52" t="str">
         <v>Landscape</v>
       </c>
       <c r="G52">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H52" t="str">
         <v>Fully Finished</v>
@@ -2072,7 +2072,7 @@
         <v>Available</v>
       </c>
       <c r="J52" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="53">
@@ -2089,13 +2089,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E53">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F53" t="str">
         <v>Pool</v>
       </c>
       <c r="G53">
-        <v>6111810</v>
+        <v>6370785</v>
       </c>
       <c r="H53" t="str">
         <v>Fully Finished</v>
@@ -2104,7 +2104,7 @@
         <v>Available</v>
       </c>
       <c r="J53" t="str">
-        <v>2br-a</v>
+        <v>2br-t3</v>
       </c>
     </row>
     <row r="54">
@@ -2121,13 +2121,13 @@
         <v>4 Bedrooms</v>
       </c>
       <c r="E54">
-        <v>179</v>
+        <v>225</v>
       </c>
       <c r="F54" t="str">
         <v>Garden</v>
       </c>
       <c r="G54">
-        <v>8988485</v>
+        <v>11298375</v>
       </c>
       <c r="H54" t="str">
         <v>Fully Finished</v>
@@ -2136,7 +2136,7 @@
         <v>Available</v>
       </c>
       <c r="J54" t="str">
-        <v>4br-a</v>
+        <v>4br-t5</v>
       </c>
     </row>
     <row r="55">
@@ -2150,16 +2150,16 @@
         <v>7th</v>
       </c>
       <c r="D55" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E55">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="F55" t="str">
         <v>Street</v>
       </c>
       <c r="G55">
-        <v>6681555</v>
+        <v>8431072</v>
       </c>
       <c r="H55" t="str">
         <v>Fully Finished</v>
@@ -2168,7 +2168,7 @@
         <v>Available</v>
       </c>
       <c r="J55" t="str">
-        <v>2br-b</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="56">
@@ -2185,13 +2185,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E56">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F56" t="str">
         <v>Street</v>
       </c>
       <c r="G56">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H56" t="str">
         <v>Fully Finished</v>
@@ -2200,7 +2200,7 @@
         <v>Available</v>
       </c>
       <c r="J56" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="57">
@@ -2217,13 +2217,13 @@
         <v>4 Bedrooms</v>
       </c>
       <c r="E57">
-        <v>179</v>
+        <v>225</v>
       </c>
       <c r="F57" t="str">
         <v>Landscape</v>
       </c>
       <c r="G57">
-        <v>8988485</v>
+        <v>11298375</v>
       </c>
       <c r="H57" t="str">
         <v>Fully Finished</v>
@@ -2232,7 +2232,7 @@
         <v>Available</v>
       </c>
       <c r="J57" t="str">
-        <v>4br-a</v>
+        <v>4br-t5</v>
       </c>
     </row>
     <row r="58">
@@ -2249,13 +2249,13 @@
         <v>4 Bedrooms</v>
       </c>
       <c r="E58">
-        <v>179</v>
+        <v>225</v>
       </c>
       <c r="F58" t="str">
         <v>Street</v>
       </c>
       <c r="G58">
-        <v>8988485</v>
+        <v>11298375</v>
       </c>
       <c r="H58" t="str">
         <v>Fully Finished</v>
@@ -2264,7 +2264,7 @@
         <v>Available</v>
       </c>
       <c r="J58" t="str">
-        <v>4br-a</v>
+        <v>4br-t5</v>
       </c>
     </row>
     <row r="59">
@@ -2278,16 +2278,16 @@
         <v>4th</v>
       </c>
       <c r="D59" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E59">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F59" t="str">
         <v>Street</v>
       </c>
       <c r="G59">
-        <v>9478811</v>
+        <v>9892355</v>
       </c>
       <c r="H59" t="str">
         <v>Fully Finished</v>
@@ -2296,7 +2296,7 @@
         <v>Available</v>
       </c>
       <c r="J59" t="str">
-        <v>3br-d</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="60">
@@ -2310,16 +2310,16 @@
         <v>1st</v>
       </c>
       <c r="D60" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E60">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F60" t="str">
         <v>Garden</v>
       </c>
       <c r="G60">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H60" t="str">
         <v>Fully Finished</v>
@@ -2328,7 +2328,7 @@
         <v>Available</v>
       </c>
       <c r="J60" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="61">
@@ -2342,16 +2342,16 @@
         <v>6th</v>
       </c>
       <c r="D61" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E61">
-        <v>124</v>
+        <v>190</v>
       </c>
       <c r="F61" t="str">
         <v>Landscape</v>
       </c>
       <c r="G61">
-        <v>6441058</v>
+        <v>9478720</v>
       </c>
       <c r="H61" t="str">
         <v>Fully Finished</v>
@@ -2360,7 +2360,7 @@
         <v>Available</v>
       </c>
       <c r="J61" t="str">
-        <v>2br-b</v>
+        <v>3br-t1</v>
       </c>
     </row>
     <row r="62">
@@ -2374,16 +2374,16 @@
         <v>7th</v>
       </c>
       <c r="D62" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E62">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="F62" t="str">
         <v>Garden</v>
       </c>
       <c r="G62">
-        <v>9478811</v>
+        <v>10043000</v>
       </c>
       <c r="H62" t="str">
         <v>Fully Finished</v>
@@ -2392,7 +2392,7 @@
         <v>Available</v>
       </c>
       <c r="J62" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="63">
@@ -2409,13 +2409,13 @@
         <v>4 Bedrooms</v>
       </c>
       <c r="E63">
-        <v>179</v>
+        <v>225</v>
       </c>
       <c r="F63" t="str">
         <v>Pool</v>
       </c>
       <c r="G63">
-        <v>8988485</v>
+        <v>11298375</v>
       </c>
       <c r="H63" t="str">
         <v>Fully Finished</v>
@@ -2424,7 +2424,7 @@
         <v>Available</v>
       </c>
       <c r="J63" t="str">
-        <v>4br-a</v>
+        <v>4br-t5</v>
       </c>
     </row>
     <row r="64">
@@ -2438,16 +2438,16 @@
         <v>3rd</v>
       </c>
       <c r="D64" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E64">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F64" t="str">
         <v>Landscape</v>
       </c>
       <c r="G64">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H64" t="str">
         <v>Fully Finished</v>
@@ -2456,7 +2456,7 @@
         <v>Available</v>
       </c>
       <c r="J64" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="65">
@@ -2470,16 +2470,16 @@
         <v>6th</v>
       </c>
       <c r="D65" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E65">
-        <v>177</v>
+        <v>226</v>
       </c>
       <c r="F65" t="str">
         <v>Landscape</v>
       </c>
       <c r="G65">
-        <v>8888055</v>
+        <v>11348590</v>
       </c>
       <c r="H65" t="str">
         <v>Fully Finished</v>
@@ -2488,7 +2488,7 @@
         <v>Available</v>
       </c>
       <c r="J65" t="str">
-        <v>3br-c</v>
+        <v>4br-t1</v>
       </c>
     </row>
     <row r="66">
@@ -2502,16 +2502,16 @@
         <v>5th</v>
       </c>
       <c r="D66" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E66">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F66" t="str">
         <v>Garden</v>
       </c>
       <c r="G66">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H66" t="str">
         <v>Fully Finished</v>
@@ -2520,7 +2520,7 @@
         <v>Available</v>
       </c>
       <c r="J66" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="67">
@@ -2534,16 +2534,16 @@
         <v>3rd</v>
       </c>
       <c r="D67" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E67">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="F67" t="str">
         <v>Pool</v>
       </c>
       <c r="G67">
-        <v>9478811</v>
+        <v>10043000</v>
       </c>
       <c r="H67" t="str">
         <v>Fully Finished</v>
@@ -2552,7 +2552,7 @@
         <v>Available</v>
       </c>
       <c r="J67" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="68">
@@ -2566,16 +2566,16 @@
         <v>5th</v>
       </c>
       <c r="D68" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E68">
-        <v>124</v>
+        <v>190</v>
       </c>
       <c r="F68" t="str">
         <v>Garden</v>
       </c>
       <c r="G68">
-        <v>6441058</v>
+        <v>9478720</v>
       </c>
       <c r="H68" t="str">
         <v>Fully Finished</v>
@@ -2584,7 +2584,7 @@
         <v>Available</v>
       </c>
       <c r="J68" t="str">
-        <v>2br-b</v>
+        <v>3br-t1</v>
       </c>
     </row>
     <row r="69">
@@ -2598,16 +2598,16 @@
         <v>2nd</v>
       </c>
       <c r="D69" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E69">
-        <v>177</v>
+        <v>222</v>
       </c>
       <c r="F69" t="str">
         <v>Street</v>
       </c>
       <c r="G69">
-        <v>8888055</v>
+        <v>11147730</v>
       </c>
       <c r="H69" t="str">
         <v>Fully Finished</v>
@@ -2616,7 +2616,7 @@
         <v>Available</v>
       </c>
       <c r="J69" t="str">
-        <v>3br-c</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="70">
@@ -2630,16 +2630,16 @@
         <v>3rd</v>
       </c>
       <c r="D70" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E70">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F70" t="str">
         <v>Garden</v>
       </c>
       <c r="G70">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H70" t="str">
         <v>Fully Finished</v>
@@ -2648,7 +2648,7 @@
         <v>Available</v>
       </c>
       <c r="J70" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="71">
@@ -2665,13 +2665,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E71">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F71" t="str">
         <v>Garden</v>
       </c>
       <c r="G71">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H71" t="str">
         <v>Fully Finished</v>
@@ -2680,7 +2680,7 @@
         <v>Available</v>
       </c>
       <c r="J71" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="72">
@@ -2694,16 +2694,16 @@
         <v>2nd</v>
       </c>
       <c r="D72" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E72">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="F72" t="str">
         <v>Pool</v>
       </c>
       <c r="G72">
-        <v>9017760</v>
+        <v>11147730</v>
       </c>
       <c r="H72" t="str">
         <v>Fully Finished</v>
@@ -2712,7 +2712,7 @@
         <v>Available</v>
       </c>
       <c r="J72" t="str">
-        <v>3br-d</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="73">
@@ -2729,13 +2729,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E73">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F73" t="str">
         <v>Garden</v>
       </c>
       <c r="G73">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H73" t="str">
         <v>Fully Finished</v>
@@ -2744,7 +2744,7 @@
         <v>Available</v>
       </c>
       <c r="J73" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="74">
@@ -2761,13 +2761,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E74">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="F74" t="str">
         <v>Landscape</v>
       </c>
       <c r="G74">
-        <v>8687195</v>
+        <v>7932192</v>
       </c>
       <c r="H74" t="str">
         <v>Fully Finished</v>
@@ -2776,7 +2776,7 @@
         <v>Available</v>
       </c>
       <c r="J74" t="str">
-        <v>3br-b</v>
+        <v>3br-t7</v>
       </c>
     </row>
     <row r="75">
@@ -2793,13 +2793,13 @@
         <v>4 Bedrooms</v>
       </c>
       <c r="E75">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="F75" t="str">
         <v>Street</v>
       </c>
       <c r="G75">
-        <v>8988485</v>
+        <v>9892355</v>
       </c>
       <c r="H75" t="str">
         <v>Fully Finished</v>
@@ -2808,7 +2808,7 @@
         <v>Available</v>
       </c>
       <c r="J75" t="str">
-        <v>4br-a</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="76">
@@ -2825,13 +2825,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E76">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="F76" t="str">
         <v>Street</v>
       </c>
       <c r="G76">
-        <v>6082163</v>
+        <v>8431072</v>
       </c>
       <c r="H76" t="str">
         <v>Fully Finished</v>
@@ -2840,7 +2840,7 @@
         <v>Available</v>
       </c>
       <c r="J76" t="str">
-        <v>3br-a</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="77">
@@ -2854,16 +2854,16 @@
         <v>1st</v>
       </c>
       <c r="D77" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E77">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="F77" t="str">
         <v>Garden</v>
       </c>
       <c r="G77">
-        <v>9478811</v>
+        <v>10043000</v>
       </c>
       <c r="H77" t="str">
         <v>Fully Finished</v>
@@ -2872,7 +2872,7 @@
         <v>Available</v>
       </c>
       <c r="J77" t="str">
-        <v>3br-d</v>
+        <v>4br-t3</v>
       </c>
     </row>
     <row r="78">
@@ -2889,13 +2889,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E78">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="F78" t="str">
         <v>Garden</v>
       </c>
       <c r="G78">
-        <v>7380720</v>
+        <v>9129504</v>
       </c>
       <c r="H78" t="str">
         <v>Fully Finished</v>
@@ -2904,7 +2904,7 @@
         <v>Available</v>
       </c>
       <c r="J78" t="str">
-        <v>3br-a</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="79">
@@ -2918,16 +2918,16 @@
         <v>4th</v>
       </c>
       <c r="D79" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E79">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="F79" t="str">
         <v>Garden</v>
       </c>
       <c r="G79">
-        <v>6681555</v>
+        <v>8431072</v>
       </c>
       <c r="H79" t="str">
         <v>Fully Finished</v>
@@ -2936,7 +2936,7 @@
         <v>Available</v>
       </c>
       <c r="J79" t="str">
-        <v>2br-b</v>
+        <v>3br-t4</v>
       </c>
     </row>
     <row r="80">
@@ -2950,16 +2950,16 @@
         <v>5th</v>
       </c>
       <c r="D80" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E80">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F80" t="str">
         <v>Garden</v>
       </c>
       <c r="G80">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H80" t="str">
         <v>Fully Finished</v>
@@ -2968,7 +2968,7 @@
         <v>Available</v>
       </c>
       <c r="J80" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="81">
@@ -2985,13 +2985,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E81">
-        <v>153</v>
+        <v>197</v>
       </c>
       <c r="F81" t="str">
         <v>Garden</v>
       </c>
       <c r="G81">
-        <v>7380720</v>
+        <v>9827936</v>
       </c>
       <c r="H81" t="str">
         <v>Fully Finished</v>
@@ -3000,7 +3000,7 @@
         <v>Available</v>
       </c>
       <c r="J81" t="str">
-        <v>3br-a</v>
+        <v>3br-t5</v>
       </c>
     </row>
     <row r="82">
@@ -3014,16 +3014,16 @@
         <v>6th</v>
       </c>
       <c r="D82" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E82">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F82" t="str">
         <v>Street</v>
       </c>
       <c r="G82">
-        <v>9478811</v>
+        <v>9892355</v>
       </c>
       <c r="H82" t="str">
         <v>Fully Finished</v>
@@ -3032,7 +3032,7 @@
         <v>Available</v>
       </c>
       <c r="J82" t="str">
-        <v>3br-d</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="83">
@@ -3046,16 +3046,16 @@
         <v>4th</v>
       </c>
       <c r="D83" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E83">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="F83" t="str">
         <v>Pool</v>
       </c>
       <c r="G83">
-        <v>9478811</v>
+        <v>9892355</v>
       </c>
       <c r="H83" t="str">
         <v>Fully Finished</v>
@@ -3064,7 +3064,7 @@
         <v>Available</v>
       </c>
       <c r="J83" t="str">
-        <v>3br-d</v>
+        <v>4br-t4</v>
       </c>
     </row>
     <row r="84">
@@ -3078,16 +3078,16 @@
         <v>7th</v>
       </c>
       <c r="D84" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E84">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F84" t="str">
         <v>Pool</v>
       </c>
       <c r="G84">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H84" t="str">
         <v>Fully Finished</v>
@@ -3096,7 +3096,7 @@
         <v>Available</v>
       </c>
       <c r="J84" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="85">
@@ -3110,16 +3110,16 @@
         <v>7th</v>
       </c>
       <c r="D85" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E85">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F85" t="str">
         <v>Garden</v>
       </c>
       <c r="G85">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H85" t="str">
         <v>Fully Finished</v>
@@ -3128,7 +3128,7 @@
         <v>Available</v>
       </c>
       <c r="J85" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
     <row r="86">
@@ -3145,13 +3145,13 @@
         <v>2 Bedrooms</v>
       </c>
       <c r="E86">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="F86" t="str">
         <v>Pool</v>
       </c>
       <c r="G86">
-        <v>6111810</v>
+        <v>7251300</v>
       </c>
       <c r="H86" t="str">
         <v>Fully Finished</v>
@@ -3160,7 +3160,7 @@
         <v>Available</v>
       </c>
       <c r="J86" t="str">
-        <v>2br-a</v>
+        <v>2br-t2</v>
       </c>
     </row>
     <row r="87">
@@ -3177,13 +3177,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E87">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="F87" t="str">
         <v>Landscape</v>
       </c>
       <c r="G87">
-        <v>7380720</v>
+        <v>9129504</v>
       </c>
       <c r="H87" t="str">
         <v>Fully Finished</v>
@@ -3192,7 +3192,7 @@
         <v>Available</v>
       </c>
       <c r="J87" t="str">
-        <v>3br-a</v>
+        <v>3br-t6</v>
       </c>
     </row>
     <row r="88">
@@ -3209,13 +3209,13 @@
         <v>3 Bedrooms</v>
       </c>
       <c r="E88">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="F88" t="str">
         <v>Pool</v>
       </c>
       <c r="G88">
-        <v>8687195</v>
+        <v>7932192</v>
       </c>
       <c r="H88" t="str">
         <v>Fully Finished</v>
@@ -3224,7 +3224,7 @@
         <v>Available</v>
       </c>
       <c r="J88" t="str">
-        <v>3br-b</v>
+        <v>3br-t7</v>
       </c>
     </row>
     <row r="89">
@@ -3238,16 +3238,16 @@
         <v>3rd</v>
       </c>
       <c r="D89" t="str">
-        <v>3 Bedrooms</v>
+        <v>4 Bedrooms</v>
       </c>
       <c r="E89">
-        <v>177</v>
+        <v>222</v>
       </c>
       <c r="F89" t="str">
         <v>Garden</v>
       </c>
       <c r="G89">
-        <v>8888055</v>
+        <v>11147730</v>
       </c>
       <c r="H89" t="str">
         <v>Fully Finished</v>
@@ -3256,7 +3256,7 @@
         <v>Available</v>
       </c>
       <c r="J89" t="str">
-        <v>3br-c</v>
+        <v>4br-t2</v>
       </c>
     </row>
     <row r="90">
@@ -3270,16 +3270,16 @@
         <v>2nd</v>
       </c>
       <c r="D90" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E90">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F90" t="str">
         <v>Garden</v>
       </c>
       <c r="G90">
-        <v>6375625</v>
+        <v>10177152</v>
       </c>
       <c r="H90" t="str">
         <v>Fully Finished</v>
@@ -3288,7 +3288,7 @@
         <v>Available</v>
       </c>
       <c r="J90" t="str">
-        <v>2br-b</v>
+        <v>3br-t2</v>
       </c>
     </row>
     <row r="91">
@@ -3302,16 +3302,16 @@
         <v>2nd</v>
       </c>
       <c r="D91" t="str">
-        <v>2 Bedrooms</v>
+        <v>3 Bedrooms</v>
       </c>
       <c r="E91">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="F91" t="str">
         <v>Pool</v>
       </c>
       <c r="G91">
-        <v>6681555</v>
+        <v>7433312</v>
       </c>
       <c r="H91" t="str">
         <v>Fully Finished</v>
@@ -3320,7 +3320,7 @@
         <v>Available</v>
       </c>
       <c r="J91" t="str">
-        <v>2br-b</v>
+        <v>3br-t3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>